<commit_message>
Tuning grid workbook: cost types and cost buckets by month, in AED and in percent
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PdcnbvMxTN9eaMqR4tfx6H
</commit_message>
<xml_diff>
--- a/output/Tuning_Grid_FY2025.xlsx
+++ b/output/Tuning_Grid_FY2025.xlsx
@@ -8,8 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning grid" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 percent is worth" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Result by month" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost types AED" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost types %" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost buckets AED" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost buckets %" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 percent is worth" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Result by month" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -63,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -73,6 +77,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -805,7 +813,6 @@
       <c r="R5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1590,6 +1597,4246 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cost type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Description (Standard v2.1)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SWNurs</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Salaries and wages — nursing (dental nurses)</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="n">
+        <v>36730.811</v>
+      </c>
+      <c r="D2" s="9" t="n">
+        <v>29995.569</v>
+      </c>
+      <c r="E2" s="9" t="n">
+        <v>32617.62</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>33952.2</v>
+      </c>
+      <c r="G2" s="9" t="n">
+        <v>40465.14</v>
+      </c>
+      <c r="H2" s="9" t="n">
+        <v>59199.4</v>
+      </c>
+      <c r="I2" s="9" t="n">
+        <v>43481.95999999999</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>47559.489</v>
+      </c>
+      <c r="K2" s="9" t="n">
+        <v>30923.731</v>
+      </c>
+      <c r="L2" s="9" t="n">
+        <v>41560.81099999999</v>
+      </c>
+      <c r="M2" s="9" t="n">
+        <v>38852.44900000001</v>
+      </c>
+      <c r="N2" s="9" t="n">
+        <v>46401.931</v>
+      </c>
+      <c r="O2" s="9" t="n">
+        <v>481741.111</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SWDoc</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Salaries and wages — medical (dentists, oral surgeons, orthodontists)</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>202921.41</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>240908</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>241587.59</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>163755.24</v>
+      </c>
+      <c r="G3" s="9" t="n">
+        <v>191193.8</v>
+      </c>
+      <c r="H3" s="9" t="n">
+        <v>232448.65</v>
+      </c>
+      <c r="I3" s="9" t="n">
+        <v>165564.06</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>155839.06</v>
+      </c>
+      <c r="K3" s="9" t="n">
+        <v>172177.1</v>
+      </c>
+      <c r="L3" s="9" t="n">
+        <v>220195.09</v>
+      </c>
+      <c r="M3" s="9" t="n">
+        <v>158753.06</v>
+      </c>
+      <c r="N3" s="9" t="n">
+        <v>246757.2</v>
+      </c>
+      <c r="O3" s="9" t="n">
+        <v>2392100.26</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SWAllied</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Salaries and wages — allied health incl. technicians (CSSD technicians; dental technicians, routed to the Prosthesis bucket)</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>20665.201</v>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>14984.34</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>16447.639</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>13193.461</v>
+      </c>
+      <c r="G4" s="9" t="n">
+        <v>17094.45</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>14851.9</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>18203.869</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>24282.36</v>
+      </c>
+      <c r="K4" s="9" t="n">
+        <v>22115.57</v>
+      </c>
+      <c r="L4" s="9" t="n">
+        <v>18079.73</v>
+      </c>
+      <c r="M4" s="9" t="n">
+        <v>20429.831</v>
+      </c>
+      <c r="N4" s="9" t="n">
+        <v>32189.55</v>
+      </c>
+      <c r="O4" s="9" t="n">
+        <v>232537.901</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SWNonClin</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Salaries and wages — non-clinical staff recorded in DIRECT cost centres (chairside assistants, clinic clerks). Admin/management in overhead cost centres go to OHF.</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Pathology laboratory supplies — none: the clinic has no laboratory (ruling 13 Oct 2026); dental lab work is Prostheses</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Imaging</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Imaging supplies (films, sensors, contrast) and outsourced imaging invoices</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Pharmacy</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Drugs, anaesthetics and pharmacy services</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>1252</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>1097</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>1063.15</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>1063.15</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>1152</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>1014</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>1506</v>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v>1359</v>
+      </c>
+      <c r="K8" s="9" t="n">
+        <v>2243.5</v>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>1145.54</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>1203.75</v>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>782.9</v>
+      </c>
+      <c r="O8" s="9" t="n">
+        <v>14881.99</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Prostheses</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Implants, abutments, bone graft; crowns, bridges, veneers, onlays, dentures and every other lab-fabricated prosthesis (in-house CAD/CAM materials and external lab invoices)</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>70074.94</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>59229.44</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>88151.42</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>70459.42</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>63639.05</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>53007.03</v>
+      </c>
+      <c r="I9" s="9" t="n">
+        <v>46524.6</v>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>69988.98</v>
+      </c>
+      <c r="K9" s="9" t="n">
+        <v>57602.32</v>
+      </c>
+      <c r="L9" s="9" t="n">
+        <v>49525.36</v>
+      </c>
+      <c r="M9" s="9" t="n">
+        <v>53926.7</v>
+      </c>
+      <c r="N9" s="9" t="n">
+        <v>68940.98</v>
+      </c>
+      <c r="O9" s="9" t="n">
+        <v>751070.24</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>All other medical, surgical and dental supplies</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>31662.751</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>28366.96</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>30966.431</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>30966.431</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>24043.48</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>23064.38</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>26049.569</v>
+      </c>
+      <c r="J10" s="9" t="n">
+        <v>30284.7</v>
+      </c>
+      <c r="K10" s="9" t="n">
+        <v>25239.34</v>
+      </c>
+      <c r="L10" s="9" t="n">
+        <v>25007.409</v>
+      </c>
+      <c r="M10" s="9" t="n">
+        <v>25059.691</v>
+      </c>
+      <c r="N10" s="9" t="n">
+        <v>23384.86</v>
+      </c>
+      <c r="O10" s="9" t="n">
+        <v>324096.002</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cleaning products/services, linen and laundry, patient food</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>All other goods and services recorded in DIRECT cost centres (e.g. rent, utilities, security if booked to the clinic rooms)</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>2258.57</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>830</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="9" t="n">
+        <v>1350</v>
+      </c>
+      <c r="M12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="O12" s="9" t="n">
+        <v>5638.57</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Depreciation</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Depreciation and amortisation recorded in DIRECT cost centres (dental chairs, imaging units)</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>10556.611</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>10556.611</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>10556.611</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>10556.611</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>10556.611</v>
+      </c>
+      <c r="H13" s="9" t="n">
+        <v>10556.611</v>
+      </c>
+      <c r="I13" s="9" t="n">
+        <v>10556.611</v>
+      </c>
+      <c r="J13" s="9" t="n">
+        <v>10556.611</v>
+      </c>
+      <c r="K13" s="9" t="n">
+        <v>10556.611</v>
+      </c>
+      <c r="L13" s="9" t="n">
+        <v>10556.611</v>
+      </c>
+      <c r="M13" s="9" t="n">
+        <v>10556.611</v>
+      </c>
+      <c r="N13" s="9" t="n">
+        <v>10556.611</v>
+      </c>
+      <c r="O13" s="9" t="n">
+        <v>126679.332</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ALL expenses of OVERHEAD cost centres except depreciation: administration, reception/front office, management, HR, finance, IT, marketing, facility rent/utilities/maintenance booked to overhead centres</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>125596.78</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>105120.36</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>120683.61</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>124341.41</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>134897.36</v>
+      </c>
+      <c r="H14" s="9" t="n">
+        <v>182451.59</v>
+      </c>
+      <c r="I14" s="9" t="n">
+        <v>140755.35</v>
+      </c>
+      <c r="J14" s="9" t="n">
+        <v>157095.1</v>
+      </c>
+      <c r="K14" s="9" t="n">
+        <v>158159.08</v>
+      </c>
+      <c r="L14" s="9" t="n">
+        <v>151280.63</v>
+      </c>
+      <c r="M14" s="9" t="n">
+        <v>157439.14</v>
+      </c>
+      <c r="N14" s="9" t="n">
+        <v>166190.4</v>
+      </c>
+      <c r="O14" s="9" t="n">
+        <v>1724010.81</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>OHDepreciation</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Depreciation and amortisation recorded in OVERHEAD cost centres</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="H15" s="9" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="I15" s="9" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="J15" s="9" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="K15" s="9" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="L15" s="9" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="M15" s="9" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="N15" s="9" t="n">
+        <v>2524.8</v>
+      </c>
+      <c r="O15" s="9" t="n">
+        <v>30297.6</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>OHC</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Overheads charged by a corporate office / shared services (group fees, head-office recharges)</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>8317</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>37300</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>62270</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>66480.95</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>2500</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>37375.73</v>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>25000</v>
+      </c>
+      <c r="J16" s="9" t="n">
+        <v>27500</v>
+      </c>
+      <c r="K16" s="9" t="n">
+        <v>28000</v>
+      </c>
+      <c r="L16" s="9" t="n">
+        <v>25500</v>
+      </c>
+      <c r="M16" s="9" t="n">
+        <v>25000</v>
+      </c>
+      <c r="N16" s="9" t="n">
+        <v>25104.5</v>
+      </c>
+      <c r="O16" s="9" t="n">
+        <v>370348.18</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NABMs</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Non-activity based mandate funding by DOH, reported as negative cost (normally 0 for a private clinic)</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr"/>
+      <c r="C18" s="10" t="n">
+        <v>511302.304</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>532341.65</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>606868.871</v>
+      </c>
+      <c r="F18" s="10" t="n">
+        <v>518123.673</v>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>488066.691</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>616494.091</v>
+      </c>
+      <c r="I18" s="10" t="n">
+        <v>480166.819</v>
+      </c>
+      <c r="J18" s="10" t="n">
+        <v>526990.1</v>
+      </c>
+      <c r="K18" s="10" t="n">
+        <v>509542.052</v>
+      </c>
+      <c r="L18" s="10" t="n">
+        <v>546725.981</v>
+      </c>
+      <c r="M18" s="10" t="n">
+        <v>493746.032</v>
+      </c>
+      <c r="N18" s="10" t="n">
+        <v>623033.732</v>
+      </c>
+      <c r="O18" s="10" t="n">
+        <v>6453401.996</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Ledger (Arjun, locked)</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr"/>
+      <c r="C19" s="10" t="n">
+        <v>511302.304</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>532341.65</v>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>606868.871</v>
+      </c>
+      <c r="F19" s="10" t="n">
+        <v>518123.673</v>
+      </c>
+      <c r="G19" s="10" t="n">
+        <v>488066.691</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>616494.091</v>
+      </c>
+      <c r="I19" s="10" t="n">
+        <v>480166.819</v>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>526990.1</v>
+      </c>
+      <c r="K19" s="10" t="n">
+        <v>509542.052</v>
+      </c>
+      <c r="L19" s="10" t="n">
+        <v>546725.981</v>
+      </c>
+      <c r="M19" s="10" t="n">
+        <v>493746.032</v>
+      </c>
+      <c r="N19" s="10" t="n">
+        <v>623033.732</v>
+      </c>
+      <c r="O19" s="10" t="n">
+        <v>6453401.996</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cost type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Description (Standard v2.1)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SWNurs</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Salaries and wages — nursing (dental nurses)</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="n">
+        <v>0.07183775764875099</v>
+      </c>
+      <c r="D2" s="11" t="n">
+        <v>0.0563464628401704</v>
+      </c>
+      <c r="E2" s="11" t="n">
+        <v>0.05374739347934029</v>
+      </c>
+      <c r="F2" s="11" t="n">
+        <v>0.065529142498764</v>
+      </c>
+      <c r="G2" s="11" t="n">
+        <v>0.08290903834697459</v>
+      </c>
+      <c r="H2" s="11" t="n">
+        <v>0.09602590010874898</v>
+      </c>
+      <c r="I2" s="11" t="n">
+        <v>0.09055594489131077</v>
+      </c>
+      <c r="J2" s="11" t="n">
+        <v>0.09024740502715327</v>
+      </c>
+      <c r="K2" s="11" t="n">
+        <v>0.0606892618158236</v>
+      </c>
+      <c r="L2" s="11" t="n">
+        <v>0.07601762572903956</v>
+      </c>
+      <c r="M2" s="11" t="n">
+        <v>0.07868913668555823</v>
+      </c>
+      <c r="N2" s="11" t="n">
+        <v>0.07447739763791796</v>
+      </c>
+      <c r="O2" s="11" t="n">
+        <v>0.07464917128959216</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SWDoc</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Salaries and wages — medical (dentists, oral surgeons, orthodontists)</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>0.3968716909986778</v>
+      </c>
+      <c r="D3" s="11" t="n">
+        <v>0.4525439630733383</v>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>0.3980886177304025</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>0.3160543486689905</v>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>0.3917370382483242</v>
+      </c>
+      <c r="H3" s="11" t="n">
+        <v>0.3770492749134882</v>
+      </c>
+      <c r="I3" s="11" t="n">
+        <v>0.3448052915126566</v>
+      </c>
+      <c r="J3" s="11" t="n">
+        <v>0.295715346455275</v>
+      </c>
+      <c r="K3" s="11" t="n">
+        <v>0.3379055748670573</v>
+      </c>
+      <c r="L3" s="11" t="n">
+        <v>0.402752196991348</v>
+      </c>
+      <c r="M3" s="11" t="n">
+        <v>0.3215277687537952</v>
+      </c>
+      <c r="N3" s="11" t="n">
+        <v>0.3960575283907742</v>
+      </c>
+      <c r="O3" s="11" t="n">
+        <v>0.3706727492697171</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SWAllied</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Salaries and wages — allied health incl. technicians (CSSD technicians; dental technicians, routed to the Prosthesis bucket)</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>0.04041679616605053</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>0.02814797602254116</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>0.02710245950315023</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>0.02546392239445118</v>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>0.03502482409724617</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>0.02409090406026293</v>
+      </c>
+      <c r="I4" s="11" t="n">
+        <v>0.03791155131858456</v>
+      </c>
+      <c r="J4" s="11" t="n">
+        <v>0.04607745003179377</v>
+      </c>
+      <c r="K4" s="11" t="n">
+        <v>0.04340283576830279</v>
+      </c>
+      <c r="L4" s="11" t="n">
+        <v>0.03306908877264422</v>
+      </c>
+      <c r="M4" s="11" t="n">
+        <v>0.04137720543747073</v>
+      </c>
+      <c r="N4" s="11" t="n">
+        <v>0.05166582216450522</v>
+      </c>
+      <c r="O4" s="11" t="n">
+        <v>0.03603338226010615</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SWNonClin</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Salaries and wages — non-clinical staff recorded in DIRECT cost centres (chairside assistants, clinic clerks). Admin/management in overhead cost centres go to OHF.</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Pathology laboratory supplies — none: the clinic has no laboratory (ruling 13 Oct 2026); dental lab work is Prostheses</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Imaging</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Imaging supplies (films, sensors, contrast) and outsourced imaging invoices</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Pharmacy</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Drugs, anaesthetics and pharmacy services</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>0.002448649243716297</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>0.002060706690900477</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>0.001751861152884871</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>0.00205192322876164</v>
+      </c>
+      <c r="G8" s="11" t="n">
+        <v>0.002360333170124081</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>0.001644784621301423</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>0.003136409973384688</v>
+      </c>
+      <c r="J8" s="11" t="n">
+        <v>0.002578796072260181</v>
+      </c>
+      <c r="K8" s="11" t="n">
+        <v>0.004402973201513111</v>
+      </c>
+      <c r="L8" s="11" t="n">
+        <v>0.002095272659083674</v>
+      </c>
+      <c r="M8" s="11" t="n">
+        <v>0.002437994276377294</v>
+      </c>
+      <c r="N8" s="11" t="n">
+        <v>0.001256593278644502</v>
+      </c>
+      <c r="O8" s="11" t="n">
+        <v>0.002306068955447728</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Prostheses</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Implants, abutments, bone graft; crowns, bridges, veneers, onlays, dentures and every other lab-fabricated prosthesis (in-house CAD/CAM materials and external lab invoices)</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>0.1370518760658665</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>0.1112620814095609</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>0.1452561240367196</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>0.1359895786888703</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>0.1303900699914799</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>0.08598140805213329</v>
+      </c>
+      <c r="I9" s="11" t="n">
+        <v>0.09689257599451077</v>
+      </c>
+      <c r="J9" s="11" t="n">
+        <v>0.1328089085544491</v>
+      </c>
+      <c r="K9" s="11" t="n">
+        <v>0.1130472348138991</v>
+      </c>
+      <c r="L9" s="11" t="n">
+        <v>0.0905853420563893</v>
+      </c>
+      <c r="M9" s="11" t="n">
+        <v>0.1092195106491509</v>
+      </c>
+      <c r="N9" s="11" t="n">
+        <v>0.1106536876882936</v>
+      </c>
+      <c r="O9" s="11" t="n">
+        <v>0.1163836129324555</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>All other medical, surgical and dental supplies</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>0.06192569591863212</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>0.05328713242707948</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>0.05102656023363571</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>0.05976648552014724</v>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>0.04926269389688796</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <v>0.03741216718328611</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>0.05425108101857409</v>
+      </c>
+      <c r="J10" s="11" t="n">
+        <v>0.05746730346547307</v>
+      </c>
+      <c r="K10" s="11" t="n">
+        <v>0.04953337982789299</v>
+      </c>
+      <c r="L10" s="11" t="n">
+        <v>0.04574029745990798</v>
+      </c>
+      <c r="M10" s="11" t="n">
+        <v>0.05075421244094171</v>
+      </c>
+      <c r="N10" s="11" t="n">
+        <v>0.03753385860013114</v>
+      </c>
+      <c r="O10" s="11" t="n">
+        <v>0.0502209535685029</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cleaning products/services, linen and laundry, patient food</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>All other goods and services recorded in DIRECT cost centres (e.g. rent, utilities, security if booked to the clinic rooms)</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>0.001955790130763815</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>0.004242707667153228</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>0.001601934138994649</v>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="11" t="n">
+        <v>0.002469244277600921</v>
+      </c>
+      <c r="M12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="11" t="n">
+        <v>0.0003210099064106532</v>
+      </c>
+      <c r="O12" s="11" t="n">
+        <v>0.0008737360547963607</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Depreciation</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Depreciation and amortisation recorded in DIRECT cost centres (dental chairs, imaging units)</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="n">
+        <v>0.02064651560811273</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>0.01983051861525395</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>0.01739520925270856</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>0.02037469343733306</v>
+      </c>
+      <c r="G13" s="11" t="n">
+        <v>0.02162944366961523</v>
+      </c>
+      <c r="H13" s="11" t="n">
+        <v>0.01712362073556355</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>0.02198529882174137</v>
+      </c>
+      <c r="J13" s="11" t="n">
+        <v>0.02003189623486286</v>
+      </c>
+      <c r="K13" s="11" t="n">
+        <v>0.02071784057579609</v>
+      </c>
+      <c r="L13" s="11" t="n">
+        <v>0.01930877874267329</v>
+      </c>
+      <c r="M13" s="11" t="n">
+        <v>0.02138064979932841</v>
+      </c>
+      <c r="N13" s="11" t="n">
+        <v>0.01694388354561836</v>
+      </c>
+      <c r="O13" s="11" t="n">
+        <v>0.01962985291765791</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>OHF</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ALL expenses of OVERHEAD cost centres except depreciation: administration, reception/front office, management, HR, finance, IT, marketing, facility rent/utilities/maintenance booked to overhead centres</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>0.2456409427797141</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>0.1974678479506535</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>0.1988627457545108</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>0.2399840356261815</v>
+      </c>
+      <c r="G14" s="11" t="n">
+        <v>0.2763912442449386</v>
+      </c>
+      <c r="H14" s="11" t="n">
+        <v>0.295950265644963</v>
+      </c>
+      <c r="I14" s="11" t="n">
+        <v>0.2931384352903402</v>
+      </c>
+      <c r="J14" s="11" t="n">
+        <v>0.298098768838352</v>
+      </c>
+      <c r="K14" s="11" t="n">
+        <v>0.3103945579745791</v>
+      </c>
+      <c r="L14" s="11" t="n">
+        <v>0.2767028369921202</v>
+      </c>
+      <c r="M14" s="11" t="n">
+        <v>0.3188666435703122</v>
+      </c>
+      <c r="N14" s="11" t="n">
+        <v>0.2667438237517451</v>
+      </c>
+      <c r="O14" s="11" t="n">
+        <v>0.267147593016612</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>OHDepreciation</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Depreciation and amortisation recorded in OVERHEAD cost centres</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>0.004937978922152481</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>0.004742818826969485</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>0.004160371573911228</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>0.004872967848353844</v>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>0.00517306353118861</v>
+      </c>
+      <c r="H15" s="11" t="n">
+        <v>0.004095416382506738</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>0.005258172576893532</v>
+      </c>
+      <c r="J15" s="11" t="n">
+        <v>0.004790981841973882</v>
+      </c>
+      <c r="K15" s="11" t="n">
+        <v>0.004955037548108002</v>
+      </c>
+      <c r="L15" s="11" t="n">
+        <v>0.004618035520064301</v>
+      </c>
+      <c r="M15" s="11" t="n">
+        <v>0.005113560082240823</v>
+      </c>
+      <c r="N15" s="11" t="n">
+        <v>0.004052429058528087</v>
+      </c>
+      <c r="O15" s="11" t="n">
+        <v>0.004694826080690356</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>OHC</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Overheads charged by a corporate office / shared services (group fees, head-office recharges)</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>0.01626630651756265</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>0.07006778447637903</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>0.1026086572827361</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>0.1283109679491522</v>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>0.005122250803220661</v>
+      </c>
+      <c r="H16" s="11" t="n">
+        <v>0.0606262582977458</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>0.05206523860200345</v>
+      </c>
+      <c r="J16" s="11" t="n">
+        <v>0.0521831434784069</v>
+      </c>
+      <c r="K16" s="11" t="n">
+        <v>0.05495130360702791</v>
+      </c>
+      <c r="L16" s="11" t="n">
+        <v>0.04664128079912851</v>
+      </c>
+      <c r="M16" s="11" t="n">
+        <v>0.05063331830482437</v>
+      </c>
+      <c r="N16" s="11" t="n">
+        <v>0.04029396597743122</v>
+      </c>
+      <c r="O16" s="11" t="n">
+        <v>0.05738805365442168</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NABMs</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Non-activity based mandate funding by DOH, reported as negative cost (normally 0 for a private clinic)</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr"/>
+      <c r="C18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cost bucket</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Description (Standard v2.1)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Allied</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Allied Health services incl. technicians</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Anaesthesia</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Anaesthesia services</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>10653.897</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>11202.858</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>11398.483</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>9130.241</v>
+      </c>
+      <c r="G3" s="9" t="n">
+        <v>10160.206</v>
+      </c>
+      <c r="H3" s="9" t="n">
+        <v>12167.191</v>
+      </c>
+      <c r="I3" s="9" t="n">
+        <v>9956.338</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>9848.518</v>
+      </c>
+      <c r="K3" s="9" t="n">
+        <v>10240.011</v>
+      </c>
+      <c r="L3" s="9" t="n">
+        <v>11107.487</v>
+      </c>
+      <c r="M3" s="9" t="n">
+        <v>9188.585999999999</v>
+      </c>
+      <c r="N3" s="9" t="n">
+        <v>11735.09</v>
+      </c>
+      <c r="O3" s="9" t="n">
+        <v>126788.906</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Dental</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Dental Services</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>365786.773</v>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>395431.569</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>438916.297</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>388573.007</v>
+      </c>
+      <c r="G4" s="9" t="n">
+        <v>355181.479</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>486496.548</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>369426.2709999999</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>387060.086</v>
+      </c>
+      <c r="K4" s="9" t="n">
+        <v>383446.4939999999</v>
+      </c>
+      <c r="L4" s="9" t="n">
+        <v>420476.6299999999</v>
+      </c>
+      <c r="M4" s="9" t="n">
+        <v>374511.97</v>
+      </c>
+      <c r="N4" s="9" t="n">
+        <v>457805.821</v>
+      </c>
+      <c r="O4" s="9" t="n">
+        <v>4823112.944999999</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Emergency department</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Home healthcare</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ICU</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Intensive / critical care</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Imaging</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Imaging services</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>17627.823</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>18425.567</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>19111.744</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>15346.808</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>17004.293</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>21397.675</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>16288.624</v>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v>16502.618</v>
+      </c>
+      <c r="K8" s="9" t="n">
+        <v>16251.931</v>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>18990.428</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>15818.889</v>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>20946.285</v>
+      </c>
+      <c r="O8" s="9" t="n">
+        <v>213712.685</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Laboratory (pathology) services</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Physician</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Physician services</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Outpatient clinics</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Operating room</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Other services</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Pharmacy</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pharmacy services</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Prosthesis</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Patient implants and prostheses</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>117233.811</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>107281.656</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>137442.347</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>105073.617</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>105720.713</v>
+      </c>
+      <c r="H15" s="9" t="n">
+        <v>96432.677</v>
+      </c>
+      <c r="I15" s="9" t="n">
+        <v>84495.58600000001</v>
+      </c>
+      <c r="J15" s="9" t="n">
+        <v>113578.878</v>
+      </c>
+      <c r="K15" s="9" t="n">
+        <v>99603.61600000001</v>
+      </c>
+      <c r="L15" s="9" t="n">
+        <v>96151.436</v>
+      </c>
+      <c r="M15" s="9" t="n">
+        <v>94226.587</v>
+      </c>
+      <c r="N15" s="9" t="n">
+        <v>132546.536</v>
+      </c>
+      <c r="O15" s="9" t="n">
+        <v>1289787.46</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SPS</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Special procedure suites</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ward</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ward services</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr"/>
+      <c r="C18" s="10" t="n">
+        <v>511302.304</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>532341.65</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>606868.8709999999</v>
+      </c>
+      <c r="F18" s="10" t="n">
+        <v>518123.673</v>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>488066.691</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>616494.091</v>
+      </c>
+      <c r="I18" s="10" t="n">
+        <v>480166.819</v>
+      </c>
+      <c r="J18" s="10" t="n">
+        <v>526990.1</v>
+      </c>
+      <c r="K18" s="10" t="n">
+        <v>509542.052</v>
+      </c>
+      <c r="L18" s="10" t="n">
+        <v>546725.9809999999</v>
+      </c>
+      <c r="M18" s="10" t="n">
+        <v>493746.0319999999</v>
+      </c>
+      <c r="N18" s="10" t="n">
+        <v>623033.732</v>
+      </c>
+      <c r="O18" s="10" t="n">
+        <v>6453401.995999999</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Ledger (Arjun, locked)</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr"/>
+      <c r="C19" s="10" t="n">
+        <v>511302.304</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>532341.65</v>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>606868.871</v>
+      </c>
+      <c r="F19" s="10" t="n">
+        <v>518123.673</v>
+      </c>
+      <c r="G19" s="10" t="n">
+        <v>488066.691</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>616494.091</v>
+      </c>
+      <c r="I19" s="10" t="n">
+        <v>480166.819</v>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>526990.1</v>
+      </c>
+      <c r="K19" s="10" t="n">
+        <v>509542.052</v>
+      </c>
+      <c r="L19" s="10" t="n">
+        <v>546725.981</v>
+      </c>
+      <c r="M19" s="10" t="n">
+        <v>493746.032</v>
+      </c>
+      <c r="N19" s="10" t="n">
+        <v>623033.732</v>
+      </c>
+      <c r="O19" s="10" t="n">
+        <v>6453401.996</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Of which overhead component (CostBucketOverheads)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Anaesthesia</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>overheads allocated to this bucket</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Dental</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>overheads allocated to this bucket</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>133926.644</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>142842.753</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>183064.738</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>190860.332</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>137224.213</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>218703.088</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>165465.043</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>183977.998</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>185520.698</v>
+      </c>
+      <c r="L23" s="4" t="n">
+        <v>176279.817</v>
+      </c>
+      <c r="M23" s="4" t="n">
+        <v>181815.157</v>
+      </c>
+      <c r="N23" s="4" t="n">
+        <v>190495.892</v>
+      </c>
+      <c r="O23" s="4" t="n">
+        <v>2090176.373</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Imaging</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>overheads allocated to this bucket</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>2511.936</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>2102.407</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>2413.672</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>2486.828</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>2697.947</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>3649.032</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>2815.107</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>3141.902</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>3163.182</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>3025.613</v>
+      </c>
+      <c r="M24" s="4" t="n">
+        <v>3148.783</v>
+      </c>
+      <c r="N24" s="4" t="n">
+        <v>3323.808</v>
+      </c>
+      <c r="O24" s="4" t="n">
+        <v>34480.217</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Prosthesis</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>overheads allocated to this bucket</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Overhead ratio</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>overhead cost types ÷ month total</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>0.2668452282194292</v>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>0.272278451254002</v>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>0.3056317746111581</v>
+      </c>
+      <c r="F26" s="8" t="n">
+        <v>0.3731679714236875</v>
+      </c>
+      <c r="G26" s="8" t="n">
+        <v>0.2866865585793479</v>
+      </c>
+      <c r="H26" s="8" t="n">
+        <v>0.3606719403252155</v>
+      </c>
+      <c r="I26" s="8" t="n">
+        <v>0.3504618464692371</v>
+      </c>
+      <c r="J26" s="8" t="n">
+        <v>0.3550728941587328</v>
+      </c>
+      <c r="K26" s="8" t="n">
+        <v>0.370300899129715</v>
+      </c>
+      <c r="L26" s="8" t="n">
+        <v>0.327962153311313</v>
+      </c>
+      <c r="M26" s="8" t="n">
+        <v>0.3746135219573774</v>
+      </c>
+      <c r="N26" s="8" t="n">
+        <v>0.3110902187877044</v>
+      </c>
+      <c r="O26" s="8" t="n">
+        <v>0.3292304727517241</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cost bucket</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Description (Standard v2.1)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Allied</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Allied Health services incl. technicians</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Anaesthesia</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Anaesthesia services</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>0.02083678660677422</v>
+      </c>
+      <c r="D3" s="11" t="n">
+        <v>0.02104448900438281</v>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>0.01878244797960645</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>0.01762174066885379</v>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>0.02081724933775495</v>
+      </c>
+      <c r="H3" s="11" t="n">
+        <v>0.01973610319648628</v>
+      </c>
+      <c r="I3" s="11" t="n">
+        <v>0.02073516454288775</v>
+      </c>
+      <c r="J3" s="11" t="n">
+        <v>0.0186882410124972</v>
+      </c>
+      <c r="K3" s="11" t="n">
+        <v>0.0200964983357252</v>
+      </c>
+      <c r="L3" s="11" t="n">
+        <v>0.02031636941724194</v>
+      </c>
+      <c r="M3" s="11" t="n">
+        <v>0.01860994398837012</v>
+      </c>
+      <c r="N3" s="11" t="n">
+        <v>0.01883540071310296</v>
+      </c>
+      <c r="O3" s="11" t="n">
+        <v>0.01964683217914943</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Dental</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Dental Services</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>0.715402160597344</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>0.7428153874490189</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>0.723247340528033</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>0.749961886030249</v>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>0.7277314464387409</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>0.7891341621958872</v>
+      </c>
+      <c r="I4" s="11" t="n">
+        <v>0.7693706778185354</v>
+      </c>
+      <c r="J4" s="11" t="n">
+        <v>0.7344731637273642</v>
+      </c>
+      <c r="K4" s="11" t="n">
+        <v>0.7525315967444429</v>
+      </c>
+      <c r="L4" s="11" t="n">
+        <v>0.7690811203647553</v>
+      </c>
+      <c r="M4" s="11" t="n">
+        <v>0.7585113514390733</v>
+      </c>
+      <c r="N4" s="11" t="n">
+        <v>0.7348010187673113</v>
+      </c>
+      <c r="O4" s="11" t="n">
+        <v>0.7473752523071552</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Emergency department</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Home healthcare</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ICU</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Intensive / critical care</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Imaging</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Imaging services</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>0.03447632225025139</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>0.03461229644533731</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>0.03149237819449796</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>0.02961997067445324</v>
+      </c>
+      <c r="G8" s="11" t="n">
+        <v>0.03484010139097978</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>0.03470864573136679</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>0.03392284380233278</v>
+      </c>
+      <c r="J8" s="11" t="n">
+        <v>0.03131485392230329</v>
+      </c>
+      <c r="K8" s="11" t="n">
+        <v>0.03189517123505246</v>
+      </c>
+      <c r="L8" s="11" t="n">
+        <v>0.03473481901347578</v>
+      </c>
+      <c r="M8" s="11" t="n">
+        <v>0.03203851367862739</v>
+      </c>
+      <c r="N8" s="11" t="n">
+        <v>0.03361982493750435</v>
+      </c>
+      <c r="O8" s="11" t="n">
+        <v>0.03311628271917124</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Laboratory (pathology) services</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Physician</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Physician services</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Outpatient clinics</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Operating room</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Other services</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Pharmacy</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pharmacy services</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Prosthesis</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Patient implants and prostheses</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>0.2292847305456304</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>0.201527827101261</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>0.2264778332978624</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>0.202796402626444</v>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>0.2166112028325244</v>
+      </c>
+      <c r="H15" s="11" t="n">
+        <v>0.1564210888762598</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>0.1759713138362441</v>
+      </c>
+      <c r="J15" s="11" t="n">
+        <v>0.2155237413378354</v>
+      </c>
+      <c r="K15" s="11" t="n">
+        <v>0.1954767336847794</v>
+      </c>
+      <c r="L15" s="11" t="n">
+        <v>0.1758676912045268</v>
+      </c>
+      <c r="M15" s="11" t="n">
+        <v>0.190840190893929</v>
+      </c>
+      <c r="N15" s="11" t="n">
+        <v>0.2127437555820814</v>
+      </c>
+      <c r="O15" s="11" t="n">
+        <v>0.199861632794524</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SPS</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Special procedure suites</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ward</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ward services</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr"/>
+      <c r="C18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>0.9999999999999998</v>
+      </c>
+      <c r="F18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>0.9999999999999998</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>0.9999999999999999</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" s="12" t="n">
+        <v>0.9999999999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1638,7 +5885,6 @@
       <c r="C2" s="5" t="n">
         <v>4817.4111</v>
       </c>
-      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1652,7 +5898,6 @@
       <c r="C3" s="5" t="n">
         <v>23921.0026</v>
       </c>
-      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1684,7 +5929,6 @@
       <c r="C5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1698,7 +5942,6 @@
       <c r="C6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1712,7 +5955,6 @@
       <c r="C7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1726,7 +5968,6 @@
       <c r="C8" s="5" t="n">
         <v>148.8199</v>
       </c>
-      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1740,7 +5981,6 @@
       <c r="C9" s="5" t="n">
         <v>7510.7024</v>
       </c>
-      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1754,7 +5994,6 @@
       <c r="C10" s="5" t="n">
         <v>3240.96</v>
       </c>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1768,7 +6007,6 @@
       <c r="C11" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1782,7 +6020,6 @@
       <c r="C12" s="5" t="n">
         <v>56.3857</v>
       </c>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1796,7 +6033,6 @@
       <c r="C13" s="5" t="n">
         <v>1266.7932</v>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1810,7 +6046,6 @@
       <c r="C14" s="5" t="n">
         <v>17240.1081</v>
       </c>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1824,7 +6059,6 @@
       <c r="C15" s="5" t="n">
         <v>302.976</v>
       </c>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1838,7 +6072,6 @@
       <c r="C16" s="5" t="n">
         <v>3703.4818</v>
       </c>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1852,14 +6085,13 @@
       <c r="C17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>